<commit_message>
Add lean cost version and break-even plans sheet with reverse solvers
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XGkqvx9XTxHdsSfBaSywkX
</commit_message>
<xml_diff>
--- a/Ke_hoach_dam_cuoi.xlsx
+++ b/Ke_hoach_dam_cuoi.xlsx
@@ -13,7 +13,8 @@
     <sheet name="Chi phí" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Hòa vốn" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Dòng tiền" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Mô phỏng" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Phương án" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Mô phỏng" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="291">
   <si>
     <t xml:space="preserve">Kế hoạch đám cưới và mô phỏng hòa vốn</t>
   </si>
@@ -73,6 +74,12 @@
   </si>
   <si>
     <t xml:space="preserve">Toàn bộ chi phí: gồm cả tiệc, nghi lễ, váy, ảnh, nhẫn. Chỉ phần tiệc: chỉ so tiền mừng với chi phí tiệc. Điểm 'lần đầu không lỗ' có thể tụt lại thành lỗ ở số khách kế tiếp vì nhà hàng tính theo bàn nguyên (bước nhảy). Dùng điểm 'an toàn' để lập kế hoạch.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phương án không lỗ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sheet Phương án so sánh kịch bản hiện tại với 3 phương án dùng bản chi phí gọn (cột L ở sheet Chi phí). Dòng 'Mừng TB mỗi phong bì tối thiểu để không lỗ' cho biết mức mừng bạn cần thực sự nhận được. Nếu mức đó cao hơn mức mừng bạn tin là có thể, phương án chưa khả thi và bạn cần cắt thêm hoặc chuẩn bị nguồn bù.</t>
   </si>
   <si>
     <t xml:space="preserve">Mẹo kiểm soát</t>
@@ -259,6 +266,9 @@
     <t xml:space="preserve">Cách tính: Cố định = trả một lần. Theo bàn = đơn giá x số bàn. Theo khách = đơn giá x số khách đến. Cột Tính: 1 = đưa vào ngân sách, 0 = tắt. Cột VAT: 1 = chịu VAT/phụ thu. Mọi đơn giá là ước tính tham khảo của Claude cho tiệc cưới tầm trung ở đô thị, hãy thay bằng báo giá thật.</t>
   </si>
   <si>
+    <t xml:space="preserve">Cột L: đơn giá của BẢN GỌN (tiệc tối giản) để sheet Phương án so sánh. Mặc định bằng giá đầy đủ nếu không cắt. Giá bản gọn là ước tính của Claude, bạn chỉnh theo thực tế. Riêng giá bàn tiệc không dùng cột này, được nhập trực tiếp ở từng phương án.</t>
+  </si>
+  <si>
     <t xml:space="preserve">STT</t>
   </si>
   <si>
@@ -290,6 +300,12 @@
   </si>
   <si>
     <t xml:space="preserve">Ghi chú / giả định</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đơn giá BẢN GỌN (VND)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chi phí hiệu dụng bản gọn (cột phụ)</t>
   </si>
   <si>
     <t xml:space="preserve">1. Tiệc cưới</t>
@@ -568,7 +584,10 @@
     <t xml:space="preserve">Theo khách chịu VAT</t>
   </si>
   <si>
-    <t xml:space="preserve">Toàn bộ chi phí</t>
+    <t xml:space="preserve">Toàn bộ chi phí (bản đầy đủ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toàn bộ chi phí (bản gọn)</t>
   </si>
   <si>
     <t xml:space="preserve">Mô phỏng hòa vốn: bao nhiêu khách đến thì không lỗ?</t>
@@ -602,6 +621,9 @@
   </si>
   <si>
     <t xml:space="preserve">Chỉ tiêu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toàn bộ chi phí</t>
   </si>
   <si>
     <t xml:space="preserve">Chỉ phần tiệc</t>
@@ -755,6 +777,111 @@
   </si>
   <si>
     <t xml:space="preserve">Cách đọc: dòng 12 là vốn tự có bạn phải gom trước, không được dựa vào tiền mừng. Nên có sẵn khoảng 60% đến 70% tổng chi phí và tránh vay thẻ tín dụng lãi cao để xoay vòng tiền cọc. Dòng 16 dương nghĩa là tiền mừng đủ trả phần quyết toán cuối, nhưng phần đã ứng trước chỉ được bù khi lãi/lỗ cuối (dòng 17) không âm.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phương án để KHÔNG LỖ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cột B là kịch bản hiện tại theo sheet Giả định. Cột C đến E là các phương án bạn chỉnh (chữ xanh). Các dòng 'tối thiểu / tối đa' tính ngược: đó là điều kiện cần để P/L bằng hoặc cao hơn mức lỗ chấp nhận ở sheet Giả định.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tham số</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hiện tại (theo Giả định)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phương án A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phương án B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phương án C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tên phương án</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Theo Giả định và Chi phí</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiệc gọn, sảnh phổ thông 4,2 triệu/bàn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiệc gọn, sảnh rẻ 3,3 triệu/bàn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giữ bàn 7 triệu, chỉ cắt cho gọn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bản chi phí (1 = đầy đủ, 2 = gọn)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tỷ lệ khách đến</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Số khách đến</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giá bàn trọn gói (VND/bàn, chưa VAT và phí phục vụ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Số người mỗi phong bì</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mừng trung bình mỗi phong bì (VND)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LÃI / (LỖ) (VND)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kết luận</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chi phí cố định hiệu dụng, đã gồm VAT, dự phòng, bàn dự phòng (VND)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tính ngược: điều kiện cần để không lỗ (giữ nguyên các tham số khác)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mừng TB mỗi phong bì TỐI THIỂU để không lỗ (VND)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giá bàn TỐI ĐA để không lỗ (VND, số âm = không khả thi)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Số khách đến xấp xỉ để hòa vốn (cố định hiệu dụng / đóng góp biên)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tham số tính toán (cột phụ, không cần chỉnh)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chi phí cố định (VND)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giá bàn mỗi bàn, gồm các khoản theo bàn khác (VND)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chi phí theo khách (VND/khách)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cố định chịu VAT (VND)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Theo bàn chịu VAT (VND/bàn)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Theo khách chịu VAT (VND/khách)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mừng từ người vắng mặt tính trên mỗi khách đến (VND)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kiểm tra: cột B khớp với sheet Hòa vốn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cách đọc: dòng 24 là mức mừng bình quân bạn phải THỰC SỰ nhận để không lỗ ở phương án đó. Nếu thấp hơn mức mừng bạn tin là có thể, phương án đó khả thi. Dòng 25 cho biết nếu giữ mức mừng, giá bàn phải xuống bao nhiêu.</t>
   </si>
   <si>
     <t xml:space="preserve">Bảng mô phỏng theo từng số khách đến (sheet phụ, không cần chỉnh)</t>
@@ -994,7 +1121,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="47">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1163,6 +1290,26 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1172,7 +1319,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="4">
     <dxf>
       <font>
         <name val="Arial"/>
@@ -1198,6 +1345,29 @@
           <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <color rgb="FF9C0006"/>
+      </font>
     </dxf>
   </dxfs>
   <colors>
@@ -1976,11 +2146,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="93860199"/>
-        <c:axId val="37700343"/>
+        <c:axId val="96059365"/>
+        <c:axId val="71637197"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="93860199"/>
+        <c:axId val="96059365"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2056,12 +2226,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="37700343"/>
+        <c:crossAx val="71637197"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="37700343"/>
+        <c:axId val="71637197"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2137,7 +2307,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="93860199"/>
+        <c:crossAx val="96059365"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2404,7 +2574,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -2464,7 +2634,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
         <v>13</v>
       </c>
@@ -2472,12 +2642,20 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="126" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>16</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="126" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -2507,17 +2685,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -2525,107 +2703,107 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B4" s="8" t="n">
         <v>300</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B5" s="11" t="n">
         <v>0.85</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B6" s="12" t="n">
         <f aca="false">ROUND(B4*B5,0)</f>
         <v>255</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B7" s="13" t="n">
         <v>10</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B8" s="13" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B9" s="13" t="n">
         <v>15</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B10" s="12" t="n">
         <f aca="false">MAX(B9,ROUNDUP(B6/B7,0)+B8)</f>
         <v>27</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
@@ -2633,64 +2811,64 @@
     </row>
     <row r="13" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B13" s="11" t="n">
         <v>0.1</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B14" s="11" t="n">
         <v>0.07</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B15" s="14" t="n">
         <f aca="false">B13+B14</f>
         <v>0.17</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B16" s="15" t="n">
         <v>0.1</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -2698,107 +2876,107 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B19" s="16" t="n">
         <v>1.4</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B20" s="8" t="n">
         <v>500000</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B21" s="15" t="n">
         <v>0.4</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B22" s="13" t="n">
         <v>300000</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B23" s="12" t="n">
         <f aca="false">(1-B5)/B5*B21*B22/B19</f>
         <v>15126.0504201681</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B24" s="13" t="n">
         <v>0</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B25" s="12" t="n">
         <f aca="false">B20/B19+B23</f>
         <v>372268.907563025</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
@@ -2806,28 +2984,28 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="9" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B29" s="13" t="n">
         <v>0</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -2846,7 +3024,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K77"/>
+  <dimension ref="A1:M78"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -2859,16 +3037,17 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B2" s="17"/>
       <c r="C2" s="17"/>
@@ -2881,39 +3060,50 @@
       <c r="J2" s="17"/>
       <c r="K2" s="17"/>
     </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
     <row r="4" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="G4" s="18" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="H4" s="18" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="I4" s="18" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="J4" s="18" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="K4" s="18" t="s">
-        <v>82</v>
+        <v>85</v>
+      </c>
+      <c r="L4" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="M4" s="18" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2921,13 +3111,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C5" s="20" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="E5" s="13" t="n">
         <v>7000000</v>
@@ -2950,7 +3140,14 @@
         <v>7000000</v>
       </c>
       <c r="K5" s="23" t="s">
-        <v>86</v>
+        <v>91</v>
+      </c>
+      <c r="L5" s="13" t="n">
+        <v>7000000</v>
+      </c>
+      <c r="M5" s="12" t="n">
+        <f aca="false">L5*F5*H5</f>
+        <v>7000000</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2958,13 +3155,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="E6" s="13" t="n">
         <v>0</v>
@@ -2987,7 +3184,14 @@
         <v>0</v>
       </c>
       <c r="K6" s="23" t="s">
-        <v>88</v>
+        <v>93</v>
+      </c>
+      <c r="L6" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="12" t="n">
+        <f aca="false">L6*F6*H6</f>
+        <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2995,13 +3199,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C7" s="20" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="E7" s="13" t="n">
         <v>150000</v>
@@ -3024,7 +3228,14 @@
         <v>150000</v>
       </c>
       <c r="K7" s="23" t="s">
-        <v>90</v>
+        <v>95</v>
+      </c>
+      <c r="L7" s="13" t="n">
+        <v>100000</v>
+      </c>
+      <c r="M7" s="12" t="n">
+        <f aca="false">L7*F7*H7</f>
+        <v>100000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3032,13 +3243,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E8" s="13" t="n">
         <v>5000000</v>
@@ -3061,7 +3272,14 @@
         <v>5000000</v>
       </c>
       <c r="K8" s="23" t="s">
-        <v>93</v>
+        <v>98</v>
+      </c>
+      <c r="L8" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="12" t="n">
+        <f aca="false">L8*F8*H8</f>
+        <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3069,13 +3287,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C9" s="20" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E9" s="13" t="n">
         <v>20000000</v>
@@ -3098,7 +3316,14 @@
         <v>20000000</v>
       </c>
       <c r="K9" s="23" t="s">
-        <v>95</v>
+        <v>100</v>
+      </c>
+      <c r="L9" s="13" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="M9" s="12" t="n">
+        <f aca="false">L9*F9*H9</f>
+        <v>10000000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3106,13 +3331,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C10" s="20" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E10" s="13" t="n">
         <v>10000000</v>
@@ -3135,19 +3360,26 @@
         <v>10000000</v>
       </c>
       <c r="K10" s="23"/>
+      <c r="L10" s="13" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="M10" s="12" t="n">
+        <f aca="false">L10*F10*H10</f>
+        <v>6000000</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="19" t="n">
         <v>7</v>
       </c>
       <c r="B11" s="20" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C11" s="20" t="s">
+        <v>102</v>
+      </c>
+      <c r="D11" s="20" t="s">
         <v>97</v>
-      </c>
-      <c r="D11" s="20" t="s">
-        <v>92</v>
       </c>
       <c r="E11" s="13" t="n">
         <v>5000000</v>
@@ -3170,7 +3402,14 @@
         <v>5000000</v>
       </c>
       <c r="K11" s="23" t="s">
-        <v>98</v>
+        <v>103</v>
+      </c>
+      <c r="L11" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="12" t="n">
+        <f aca="false">L11*F11*H11</f>
+        <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3178,13 +3417,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="20" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C12" s="20" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E12" s="13" t="n">
         <v>4000000</v>
@@ -3207,19 +3446,26 @@
         <v>4000000</v>
       </c>
       <c r="K12" s="23"/>
+      <c r="L12" s="13" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="M12" s="12" t="n">
+        <f aca="false">L12*F12*H12</f>
+        <v>2000000</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="19" t="n">
         <v>9</v>
       </c>
       <c r="B13" s="20" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E13" s="13" t="n">
         <v>3000000</v>
@@ -3242,19 +3488,26 @@
         <v>3000000</v>
       </c>
       <c r="K13" s="23"/>
+      <c r="L13" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="12" t="n">
+        <f aca="false">L13*F13*H13</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="19" t="n">
         <v>10</v>
       </c>
       <c r="B14" s="20" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C14" s="20" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="D14" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E14" s="13" t="n">
         <v>500000</v>
@@ -3277,19 +3530,26 @@
         <v>500000</v>
       </c>
       <c r="K14" s="23"/>
+      <c r="L14" s="13" t="n">
+        <v>300000</v>
+      </c>
+      <c r="M14" s="12" t="n">
+        <f aca="false">L14*F14*H14</f>
+        <v>300000</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="19" t="n">
         <v>11</v>
       </c>
       <c r="B15" s="20" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C15" s="20" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E15" s="13" t="n">
         <v>3000000</v>
@@ -3312,7 +3572,14 @@
         <v>3000000</v>
       </c>
       <c r="K15" s="23" t="s">
-        <v>103</v>
+        <v>108</v>
+      </c>
+      <c r="L15" s="13" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="M15" s="12" t="n">
+        <f aca="false">L15*F15*H15</f>
+        <v>1000000</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3320,13 +3587,13 @@
         <v>12</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C16" s="20" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="D16" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E16" s="13" t="n">
         <v>2000000</v>
@@ -3349,19 +3616,26 @@
         <v>2000000</v>
       </c>
       <c r="K16" s="23"/>
+      <c r="L16" s="13" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="M16" s="12" t="n">
+        <f aca="false">L16*F16*H16</f>
+        <v>1500000</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="19" t="n">
         <v>13</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C17" s="20" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="D17" s="20" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="E17" s="13" t="n">
         <v>25000</v>
@@ -3384,7 +3658,14 @@
         <v>25000</v>
       </c>
       <c r="K17" s="23" t="s">
-        <v>107</v>
+        <v>112</v>
+      </c>
+      <c r="L17" s="13" t="n">
+        <v>15000</v>
+      </c>
+      <c r="M17" s="12" t="n">
+        <f aca="false">L17*F17*H17</f>
+        <v>15000</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3392,13 +3673,13 @@
         <v>14</v>
       </c>
       <c r="B18" s="20" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C18" s="20" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="D18" s="20" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="E18" s="13" t="n">
         <v>12000</v>
@@ -3421,7 +3702,14 @@
         <v>8400</v>
       </c>
       <c r="K18" s="23" t="s">
-        <v>109</v>
+        <v>114</v>
+      </c>
+      <c r="L18" s="13" t="n">
+        <v>8000</v>
+      </c>
+      <c r="M18" s="12" t="n">
+        <f aca="false">L18*F18*H18</f>
+        <v>5600</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3429,13 +3717,13 @@
         <v>15</v>
       </c>
       <c r="B19" s="20" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="C19" s="20" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="D19" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E19" s="13" t="n">
         <v>15000000</v>
@@ -3458,7 +3746,14 @@
         <v>15000000</v>
       </c>
       <c r="K19" s="23" t="s">
-        <v>112</v>
+        <v>117</v>
+      </c>
+      <c r="L19" s="13" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="M19" s="12" t="n">
+        <f aca="false">L19*F19*H19</f>
+        <v>10000000</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3466,13 +3761,13 @@
         <v>16</v>
       </c>
       <c r="B20" s="20" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="C20" s="20" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="D20" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E20" s="13" t="n">
         <v>3000000</v>
@@ -3495,7 +3790,14 @@
         <v>15000000</v>
       </c>
       <c r="K20" s="23" t="s">
-        <v>114</v>
+        <v>119</v>
+      </c>
+      <c r="L20" s="13" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="M20" s="12" t="n">
+        <f aca="false">L20*F20*H20</f>
+        <v>9000000</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3503,13 +3805,13 @@
         <v>17</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="C21" s="20" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="D21" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E21" s="13" t="n">
         <v>5000000</v>
@@ -3532,19 +3834,26 @@
         <v>5000000</v>
       </c>
       <c r="K21" s="23"/>
+      <c r="L21" s="13" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="M21" s="12" t="n">
+        <f aca="false">L21*F21*H21</f>
+        <v>2000000</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="19" t="n">
         <v>18</v>
       </c>
       <c r="B22" s="20" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="C22" s="20" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="D22" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E22" s="13" t="n">
         <v>4000000</v>
@@ -3567,19 +3876,26 @@
         <v>4000000</v>
       </c>
       <c r="K22" s="23"/>
+      <c r="L22" s="13" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="M22" s="12" t="n">
+        <f aca="false">L22*F22*H22</f>
+        <v>2000000</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="19" t="n">
         <v>19</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="C23" s="20" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="D23" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E23" s="13" t="n">
         <v>3000000</v>
@@ -3602,7 +3918,14 @@
         <v>3000000</v>
       </c>
       <c r="K23" s="23" t="s">
-        <v>118</v>
+        <v>123</v>
+      </c>
+      <c r="L23" s="13" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="M23" s="12" t="n">
+        <f aca="false">L23*F23*H23</f>
+        <v>2000000</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3610,13 +3933,13 @@
         <v>20</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="C24" s="20" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="D24" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E24" s="13" t="n">
         <v>4000000</v>
@@ -3639,19 +3962,26 @@
         <v>4000000</v>
       </c>
       <c r="K24" s="23"/>
+      <c r="L24" s="13" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="M24" s="12" t="n">
+        <f aca="false">L24*F24*H24</f>
+        <v>2000000</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="19" t="n">
         <v>21</v>
       </c>
       <c r="B25" s="20" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="C25" s="20" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="D25" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E25" s="13" t="n">
         <v>12000000</v>
@@ -3674,19 +4004,26 @@
         <v>12000000</v>
       </c>
       <c r="K25" s="23"/>
+      <c r="L25" s="13" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="M25" s="12" t="n">
+        <f aca="false">L25*F25*H25</f>
+        <v>6000000</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="19" t="n">
         <v>22</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="C26" s="20" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D26" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E26" s="13" t="n">
         <v>4000000</v>
@@ -3709,19 +4046,26 @@
         <v>4000000</v>
       </c>
       <c r="K26" s="23"/>
+      <c r="L26" s="13" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="M26" s="12" t="n">
+        <f aca="false">L26*F26*H26</f>
+        <v>2000000</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="19" t="n">
         <v>23</v>
       </c>
       <c r="B27" s="20" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="C27" s="20" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="D27" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E27" s="13" t="n">
         <v>3000000</v>
@@ -3744,19 +4088,26 @@
         <v>3000000</v>
       </c>
       <c r="K27" s="23"/>
+      <c r="L27" s="13" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="M27" s="12" t="n">
+        <f aca="false">L27*F27*H27</f>
+        <v>1500000</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="19" t="n">
         <v>24</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="C28" s="20" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="D28" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E28" s="13" t="n">
         <v>6000000</v>
@@ -3779,19 +4130,26 @@
         <v>6000000</v>
       </c>
       <c r="K28" s="23"/>
+      <c r="L28" s="13" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="M28" s="12" t="n">
+        <f aca="false">L28*F28*H28</f>
+        <v>4000000</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="19" t="n">
         <v>25</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="C29" s="20" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="D29" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E29" s="13" t="n">
         <v>2500000</v>
@@ -3814,19 +4172,26 @@
         <v>2500000</v>
       </c>
       <c r="K29" s="23"/>
+      <c r="L29" s="13" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="M29" s="12" t="n">
+        <f aca="false">L29*F29*H29</f>
+        <v>1500000</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="19" t="n">
         <v>26</v>
       </c>
       <c r="B30" s="20" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="C30" s="20" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="D30" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E30" s="13" t="n">
         <v>1500000</v>
@@ -3849,19 +4214,26 @@
         <v>1500000</v>
       </c>
       <c r="K30" s="23"/>
+      <c r="L30" s="13" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="M30" s="12" t="n">
+        <f aca="false">L30*F30*H30</f>
+        <v>1000000</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="19" t="n">
         <v>27</v>
       </c>
       <c r="B31" s="20" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="C31" s="20" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="D31" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E31" s="13" t="n">
         <v>1500000</v>
@@ -3884,19 +4256,26 @@
         <v>1500000</v>
       </c>
       <c r="K31" s="23"/>
+      <c r="L31" s="13" t="n">
+        <v>800000</v>
+      </c>
+      <c r="M31" s="12" t="n">
+        <f aca="false">L31*F31*H31</f>
+        <v>800000</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="19" t="n">
         <v>28</v>
       </c>
       <c r="B32" s="20" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="C32" s="20" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="D32" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E32" s="13" t="n">
         <v>12000000</v>
@@ -3919,19 +4298,26 @@
         <v>12000000</v>
       </c>
       <c r="K32" s="23"/>
+      <c r="L32" s="13" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="M32" s="12" t="n">
+        <f aca="false">L32*F32*H32</f>
+        <v>6000000</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="19" t="n">
         <v>29</v>
       </c>
       <c r="B33" s="20" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="C33" s="20" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="D33" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E33" s="13" t="n">
         <v>8000000</v>
@@ -3954,19 +4340,26 @@
         <v>8000000</v>
       </c>
       <c r="K33" s="23"/>
+      <c r="L33" s="13" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="M33" s="12" t="n">
+        <f aca="false">L33*F33*H33</f>
+        <v>5000000</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="19" t="n">
         <v>30</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="C34" s="20" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="D34" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E34" s="13" t="n">
         <v>8000000</v>
@@ -3989,19 +4382,26 @@
         <v>8000000</v>
       </c>
       <c r="K34" s="23"/>
+      <c r="L34" s="13" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="M34" s="12" t="n">
+        <f aca="false">L34*F34*H34</f>
+        <v>4000000</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="19" t="n">
         <v>31</v>
       </c>
       <c r="B35" s="20" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="C35" s="20" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="D35" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E35" s="13" t="n">
         <v>2000000</v>
@@ -4024,19 +4424,26 @@
         <v>2000000</v>
       </c>
       <c r="K35" s="23"/>
+      <c r="L35" s="13" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="M35" s="12" t="n">
+        <f aca="false">L35*F35*H35</f>
+        <v>1000000</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="19" t="n">
         <v>32</v>
       </c>
       <c r="B36" s="20" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="C36" s="20" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="D36" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E36" s="13" t="n">
         <v>10000000</v>
@@ -4059,7 +4466,14 @@
         <v>10000000</v>
       </c>
       <c r="K36" s="23" t="s">
-        <v>135</v>
+        <v>140</v>
+      </c>
+      <c r="L36" s="13" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="M36" s="12" t="n">
+        <f aca="false">L36*F36*H36</f>
+        <v>6000000</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4067,13 +4481,13 @@
         <v>33</v>
       </c>
       <c r="B37" s="20" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="C37" s="20" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="D37" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E37" s="13" t="n">
         <v>1000000</v>
@@ -4096,19 +4510,26 @@
         <v>1000000</v>
       </c>
       <c r="K37" s="23"/>
+      <c r="L37" s="13" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="M37" s="12" t="n">
+        <f aca="false">L37*F37*H37</f>
+        <v>1000000</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="19" t="n">
         <v>34</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C38" s="20" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="D38" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E38" s="13" t="n">
         <v>5000000</v>
@@ -4131,19 +4552,26 @@
         <v>5000000</v>
       </c>
       <c r="K38" s="23"/>
+      <c r="L38" s="13" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="M38" s="12" t="n">
+        <f aca="false">L38*F38*H38</f>
+        <v>3000000</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="19" t="n">
         <v>35</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C39" s="20" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="D39" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E39" s="13" t="n">
         <v>2000000</v>
@@ -4166,19 +4594,26 @@
         <v>2000000</v>
       </c>
       <c r="K39" s="23"/>
+      <c r="L39" s="13" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="M39" s="12" t="n">
+        <f aca="false">L39*F39*H39</f>
+        <v>1000000</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="19" t="n">
         <v>36</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C40" s="20" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="D40" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E40" s="13" t="n">
         <v>1000000</v>
@@ -4201,7 +4636,14 @@
         <v>1000000</v>
       </c>
       <c r="K40" s="23" t="s">
-        <v>141</v>
+        <v>146</v>
+      </c>
+      <c r="L40" s="13" t="n">
+        <v>500000</v>
+      </c>
+      <c r="M40" s="12" t="n">
+        <f aca="false">L40*F40*H40</f>
+        <v>500000</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4209,13 +4651,13 @@
         <v>37</v>
       </c>
       <c r="B41" s="20" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C41" s="20" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="D41" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E41" s="13" t="n">
         <v>500000</v>
@@ -4238,19 +4680,26 @@
         <v>500000</v>
       </c>
       <c r="K41" s="23"/>
+      <c r="L41" s="13" t="n">
+        <v>200000</v>
+      </c>
+      <c r="M41" s="12" t="n">
+        <f aca="false">L41*F41*H41</f>
+        <v>200000</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="19" t="n">
         <v>38</v>
       </c>
       <c r="B42" s="20" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C42" s="20" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="D42" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E42" s="13" t="n">
         <v>2000000</v>
@@ -4273,19 +4722,26 @@
         <v>2000000</v>
       </c>
       <c r="K42" s="23"/>
+      <c r="L42" s="13" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="M42" s="12" t="n">
+        <f aca="false">L42*F42*H42</f>
+        <v>1000000</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="19" t="n">
         <v>39</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="C43" s="20" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="D43" s="20" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="E43" s="13" t="n">
         <v>150000</v>
@@ -4308,7 +4764,14 @@
         <v>0</v>
       </c>
       <c r="K43" s="23" t="s">
-        <v>146</v>
+        <v>151</v>
+      </c>
+      <c r="L43" s="13" t="n">
+        <v>150000</v>
+      </c>
+      <c r="M43" s="12" t="n">
+        <f aca="false">L43*F43*H43</f>
+        <v>0</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4316,13 +4779,13 @@
         <v>40</v>
       </c>
       <c r="B44" s="20" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="C44" s="20" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="D44" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E44" s="13" t="n">
         <v>3000000</v>
@@ -4345,7 +4808,14 @@
         <v>0</v>
       </c>
       <c r="K44" s="23" t="s">
-        <v>148</v>
+        <v>153</v>
+      </c>
+      <c r="L44" s="13" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="M44" s="12" t="n">
+        <f aca="false">L44*F44*H44</f>
+        <v>0</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4353,13 +4823,13 @@
         <v>41</v>
       </c>
       <c r="B45" s="20" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="C45" s="20" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="D45" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E45" s="13" t="n">
         <v>8000000</v>
@@ -4382,7 +4852,14 @@
         <v>0</v>
       </c>
       <c r="K45" s="23" t="s">
-        <v>150</v>
+        <v>155</v>
+      </c>
+      <c r="L45" s="13" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="M45" s="12" t="n">
+        <f aca="false">L45*F45*H45</f>
+        <v>0</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4390,13 +4867,13 @@
         <v>42</v>
       </c>
       <c r="B46" s="20" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="C46" s="20" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="D46" s="20" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="E46" s="13" t="n">
         <v>4500000</v>
@@ -4419,7 +4896,14 @@
         <v>0</v>
       </c>
       <c r="K46" s="23" t="s">
-        <v>152</v>
+        <v>157</v>
+      </c>
+      <c r="L46" s="13" t="n">
+        <v>4500000</v>
+      </c>
+      <c r="M46" s="12" t="n">
+        <f aca="false">L46*F46*H46</f>
+        <v>0</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4427,13 +4911,13 @@
         <v>43</v>
       </c>
       <c r="B47" s="20" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="C47" s="20" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="D47" s="20" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E47" s="13" t="n">
         <v>30000000</v>
@@ -4456,7 +4940,14 @@
         <v>0</v>
       </c>
       <c r="K47" s="23" t="s">
-        <v>154</v>
+        <v>159</v>
+      </c>
+      <c r="L47" s="13" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="M47" s="12" t="n">
+        <f aca="false">L47*F47*H47</f>
+        <v>0</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4477,7 +4968,12 @@
         <v>0</v>
       </c>
       <c r="K48" s="19" t="s">
-        <v>155</v>
+        <v>160</v>
+      </c>
+      <c r="L48" s="13"/>
+      <c r="M48" s="12" t="n">
+        <f aca="false">L48*F48*H48</f>
+        <v>0</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4498,6 +4994,11 @@
         <v>0</v>
       </c>
       <c r="K49" s="24"/>
+      <c r="L49" s="13"/>
+      <c r="M49" s="12" t="n">
+        <f aca="false">L49*F49*H49</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="19"/>
@@ -4517,6 +5018,11 @@
         <v>0</v>
       </c>
       <c r="K50" s="24"/>
+      <c r="L50" s="13"/>
+      <c r="M50" s="12" t="n">
+        <f aca="false">L50*F50*H50</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="19"/>
@@ -4536,6 +5042,11 @@
         <v>0</v>
       </c>
       <c r="K51" s="24"/>
+      <c r="L51" s="13"/>
+      <c r="M51" s="12" t="n">
+        <f aca="false">L51*F51*H51</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="19"/>
@@ -4555,6 +5066,11 @@
         <v>0</v>
       </c>
       <c r="K52" s="24"/>
+      <c r="L52" s="13"/>
+      <c r="M52" s="12" t="n">
+        <f aca="false">L52*F52*H52</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="19"/>
@@ -4574,10 +5090,15 @@
         <v>0</v>
       </c>
       <c r="K53" s="24"/>
+      <c r="L53" s="13"/>
+      <c r="M53" s="12" t="n">
+        <f aca="false">L53*F53*H53</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="B55" s="6"/>
       <c r="C55" s="6"/>
@@ -4592,7 +5113,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C56" s="7" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="I56" s="25" t="n">
         <f aca="false">SUM(I5:I53)</f>
@@ -4601,7 +5122,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C57" s="7" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="I57" s="25" t="n">
         <f aca="false">'Giả định'!$B$15*SUMPRODUCT($G$5:$G$53,$I$5:$I$53)</f>
@@ -4610,7 +5131,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C58" s="7" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="I58" s="25" t="n">
         <f aca="false">'Giả định'!$B$16*(I56+I57)</f>
@@ -4619,7 +5140,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C59" s="26" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="D59" s="27"/>
       <c r="E59" s="27"/>
@@ -4633,7 +5154,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C60" s="7" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="I60" s="25" t="n">
         <f aca="false">'Giả định'!$B$6/'Giả định'!$B$19*'Giả định'!$B$20+'Giả định'!$B$6*'Giả định'!$B$23+'Giả định'!$B$24</f>
@@ -4642,7 +5163,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C61" s="26" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="D61" s="27"/>
       <c r="E61" s="27"/>
@@ -4656,7 +5177,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="5" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="B63" s="6"/>
       <c r="C63" s="6"/>
@@ -4671,18 +5192,18 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C64" s="29" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I64" s="30" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="J64" s="30" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C65" s="7" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="I65" s="25" t="n">
         <f aca="false">SUMIFS($I$5:$I$53,$B$5:$B$53,C65)</f>
@@ -4695,7 +5216,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C66" s="7" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="I66" s="25" t="n">
         <f aca="false">SUMIFS($I$5:$I$53,$B$5:$B$53,C66)</f>
@@ -4708,7 +5229,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C67" s="7" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="I67" s="25" t="n">
         <f aca="false">SUMIFS($I$5:$I$53,$B$5:$B$53,C67)</f>
@@ -4721,7 +5242,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C68" s="7" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="I68" s="25" t="n">
         <f aca="false">SUMIFS($I$5:$I$53,$B$5:$B$53,C68)</f>
@@ -4734,7 +5255,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C69" s="7" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="I69" s="25" t="n">
         <f aca="false">SUMIFS($I$5:$I$53,$B$5:$B$53,C69)</f>
@@ -4747,7 +5268,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C70" s="7" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="I70" s="25" t="n">
         <f aca="false">SUMIFS($I$5:$I$53,$B$5:$B$53,C70)</f>
@@ -4760,7 +5281,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C71" s="7" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="I71" s="25" t="n">
         <f aca="false">SUMIFS($I$5:$I$53,$B$5:$B$53,C71)</f>
@@ -4773,7 +5294,7 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C72" s="9" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="I72" s="9" t="str">
         <f aca="false">IF(ABS(SUM(I65:I71)-I56)&lt;1,"OK","LỆCH: có hạng mục sai tên nhóm")</f>
@@ -4782,7 +5303,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="5" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="B74" s="6"/>
       <c r="C74" s="6"/>
@@ -4797,30 +5318,30 @@
     </row>
     <row r="75" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B75" s="30" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="C75" s="30" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D75" s="30" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="E75" s="30" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="F75" s="30" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="G75" s="30" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="H75" s="30" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B76" s="7" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C76" s="25" t="n">
         <f aca="false">SUMIFS($J$5:$J$53,$B$5:$B$53,$B$76,$D$5:$D$53,"Cố định")</f>
@@ -4849,7 +5370,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B77" s="7" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="C77" s="25" t="n">
         <f aca="false">SUMIFS($J$5:$J$53,$D$5:$D$53,"Cố định")</f>
@@ -4873,6 +5394,35 @@
       </c>
       <c r="H77" s="25" t="n">
         <f aca="false">SUMIFS($J$5:$J$53,$D$5:$D$53,"Theo khách",$G$5:$G$53,1)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B78" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="C78" s="25" t="n">
+        <f aca="false">SUMIFS($M$5:$M$53,$D$5:$D$53,"Cố định")</f>
+        <v>93300000</v>
+      </c>
+      <c r="D78" s="25" t="n">
+        <f aca="false">SUMIFS($M$5:$M$53,$D$5:$D$53,"Theo bàn")</f>
+        <v>7100000</v>
+      </c>
+      <c r="E78" s="25" t="n">
+        <f aca="false">SUMIFS($M$5:$M$53,$D$5:$D$53,"Theo khách")</f>
+        <v>20600</v>
+      </c>
+      <c r="F78" s="25" t="n">
+        <f aca="false">SUMIFS($M$5:$M$53,$D$5:$D$53,"Cố định",$G$5:$G$53,1)</f>
+        <v>9000000</v>
+      </c>
+      <c r="G78" s="25" t="n">
+        <f aca="false">SUMIFS($M$5:$M$53,$D$5:$D$53,"Theo bàn",$G$5:$G$53,1)</f>
+        <v>7000000</v>
+      </c>
+      <c r="H78" s="25" t="n">
+        <f aca="false">SUMIFS($M$5:$M$53,$D$5:$D$53,"Theo khách",$G$5:$G$53,1)</f>
         <v>0</v>
       </c>
     </row>
@@ -4914,24 +5464,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B5" s="32" t="n">
         <f aca="false">'Giả định'!$B$4</f>
@@ -4940,7 +5490,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B6" s="32" t="n">
         <f aca="false">'Giả định'!$B$6</f>
@@ -4949,7 +5499,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B7" s="32" t="n">
         <f aca="false">'Giả định'!$B$10</f>
@@ -4958,7 +5508,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="B8" s="32" t="n">
         <f aca="false">'Chi phí'!I59</f>
@@ -4967,7 +5517,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="B9" s="32" t="n">
         <f aca="false">'Chi phí'!I60</f>
@@ -4976,7 +5526,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="33" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="B10" s="28" t="n">
         <f aca="false">B9-B8</f>
@@ -4985,7 +5535,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="B11" s="12" t="n">
         <f aca="false">IF(B6=0,0,B8/B6)</f>
@@ -4994,7 +5544,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="B12" s="32" t="n">
         <f aca="false">'Giả định'!$B$20/'Giả định'!$B$19+'Giả định'!$B$23</f>
@@ -5003,7 +5553,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="B13" s="32" t="n">
         <f aca="false">INDEX('Mô phỏng'!$G$5:$G$1005,B6+1)</f>
@@ -5012,25 +5562,25 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="29" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="B16" s="30" t="s">
-        <v>175</v>
+        <v>193</v>
       </c>
       <c r="C16" s="30" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="B17" s="12" t="str">
         <f aca="false">IF(COUNT('Mô phỏng'!$H$5:$H$1005)=0,"Không đạt (trên 1,000)",MIN('Mô phỏng'!$H$5:$H$1005))</f>
@@ -5043,7 +5593,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="33" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="B18" s="34" t="str">
         <f aca="false">IF(COUNTIF('Mô phỏng'!$F$5:$F$1005,"&lt;0")=0,0,IF(MAX('Mô phỏng'!$I$5:$I$1005)&gt;=1000,"Không đạt (trên 1,000)",MAX('Mô phỏng'!$I$5:$I$1005)+1))</f>
@@ -5056,7 +5606,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="B19" s="12" t="str">
         <f aca="false">IF(ISNUMBER(B18),ROUNDUP(B18/'Giả định'!$B$5,0),"n/a")</f>
@@ -5069,7 +5619,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="B20" s="12" t="str">
         <f aca="false">IF(ISNUMBER(B18),INDEX('Mô phỏng'!$B$5:$B$1005,B18+1),"n/a")</f>
@@ -5082,7 +5632,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="33" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="B21" s="34" t="n">
         <f aca="false">IF(B6=0,0,(INDEX('Mô phỏng'!$D$5:$D$1005,B6+1)-'Giả định'!$B$24-B6*'Giả định'!$B$23)/(B6/'Giả định'!$B$19))</f>
@@ -5095,7 +5645,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="B22" s="12" t="n">
         <f aca="false">B21/'Giả định'!$B$19</f>
@@ -5108,7 +5658,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="B23" s="12" t="n">
         <f aca="false">'Giả định'!$B$20/'Giả định'!$B$19+'Giả định'!$B$23-(('Chi phí'!$D$77+'Giả định'!$B$15*'Chi phí'!$G$77)/'Giả định'!$B$7+'Chi phí'!$E$77+'Giả định'!$B$15*'Chi phí'!$H$77)*(1+'Giả định'!$B$16)</f>
@@ -5121,7 +5671,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="B24" s="12" t="str">
         <f aca="false">IF(B23&lt;=0,"Không bao giờ hòa vốn",MAX(0,('Chi phí'!$C$77+'Giả định'!$B$15*'Chi phí'!$F$77+'Giả định'!$B$8*('Chi phí'!$D$77+'Giả định'!$B$15*'Chi phí'!$G$77))*(1+'Giả định'!$B$16)-'Giả định'!$B$24)/B23)</f>
@@ -5134,7 +5684,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="B25" s="9" t="str">
         <f aca="false">IF(ABS(B8-INDEX('Mô phỏng'!$D$5:$D$1005,B6+1))&lt;1,"OK","LỆCH")</f>
@@ -5143,12 +5693,12 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="B28" s="6"/>
       <c r="C28" s="6"/>
@@ -5159,7 +5709,7 @@
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="30" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="B29" s="35" t="n">
         <v>500000</v>
@@ -5501,7 +6051,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="B42" s="6"/>
       <c r="C42" s="6"/>
@@ -5512,7 +6062,7 @@
     </row>
     <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="30" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="B43" s="35" t="n">
         <v>500000</v>
@@ -5854,7 +6404,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="B56" s="6"/>
       <c r="C56" s="6"/>
@@ -5865,7 +6415,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="B57" s="32" t="n">
         <f aca="false">'Chi phí'!$E$5</f>
@@ -5874,7 +6424,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="33" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="B58" s="34" t="n">
         <f aca="false">IFERROR('Chi phí'!$E$5+(B10+'Giả định'!$B$29)/('Giả định'!$B$10*'Chi phí'!$F$5*'Chi phí'!$H$5*(1+'Giả định'!$B$15*'Chi phí'!$G$5)*(1+'Giả định'!$B$16)),"n/a")</f>
@@ -5883,7 +6433,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="33" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="B59" s="34" t="str">
         <f aca="false">IF('Giả định'!$B$28="","Chưa nhập ngân sách trần",IFERROR('Chi phí'!$E$5+('Giả định'!$B$28-B8)/('Giả định'!$B$10*'Chi phí'!$F$5*'Chi phí'!$H$5*(1+'Giả định'!$B$15*'Chi phí'!$G$5)*(1+'Giả định'!$B$16)),"n/a"))</f>
@@ -5892,12 +6442,12 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="9" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="30" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="B61" s="35" t="n">
         <v>500000</v>
@@ -6123,12 +6673,12 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="9" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="5" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="B71" s="6"/>
       <c r="C71" s="6"/>
@@ -6139,19 +6689,19 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="30" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="B72" s="30" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="C72" s="30" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="D72" s="30" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
       <c r="E72" s="30" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6754,40 +7304,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="37" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="C5" s="15" t="n">
         <v>0.1</v>
@@ -6806,10 +7356,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="37" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="C6" s="15" t="n">
         <v>0.3</v>
@@ -6828,10 +7378,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="37" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="C7" s="15" t="n">
         <v>0.25</v>
@@ -6850,10 +7400,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="37" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="C8" s="15" t="n">
         <v>0.35</v>
@@ -6872,7 +7422,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="26" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="C9" s="38" t="n">
         <f aca="false">SUM(C5:C8)</f>
@@ -6889,7 +7439,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
@@ -6899,7 +7449,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="33" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="B12" s="34" t="n">
         <f aca="false">SUMPRODUCT(D5:D8,F5:F8)</f>
@@ -6908,7 +7458,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="B13" s="14" t="n">
         <f aca="false">IF(D9=0,0,B12/D9)</f>
@@ -6917,7 +7467,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="B14" s="12" t="n">
         <f aca="false">D9-B12</f>
@@ -6926,7 +7476,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="B15" s="32" t="n">
         <f aca="false">'Chi phí'!$I$60</f>
@@ -6935,7 +7485,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="B16" s="12" t="n">
         <f aca="false">B15-B14</f>
@@ -6944,7 +7494,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="33" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="B17" s="40" t="n">
         <f aca="false">B15-D9</f>
@@ -6953,7 +7503,7 @@
     </row>
     <row r="19" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="41" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="B19" s="41"/>
       <c r="C19" s="41"/>
@@ -6986,6 +7536,628 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:E38"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="26"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="29" t="s">
+        <v>247</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>248</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>249</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>250</v>
+      </c>
+      <c r="E4" s="18" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
+        <v>252</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>253</v>
+      </c>
+      <c r="C5" s="42" t="s">
+        <v>254</v>
+      </c>
+      <c r="D5" s="42" t="s">
+        <v>255</v>
+      </c>
+      <c r="E5" s="42" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="B6" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="22" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="32" t="n">
+        <f aca="false">'Giả định'!$B$4</f>
+        <v>300</v>
+      </c>
+      <c r="C7" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="D7" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="E7" s="13" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="s">
+        <v>258</v>
+      </c>
+      <c r="B8" s="44" t="n">
+        <f aca="false">'Giả định'!$B$5</f>
+        <v>0.85</v>
+      </c>
+      <c r="C8" s="44" t="n">
+        <f aca="false">'Giả định'!$B$5</f>
+        <v>0.85</v>
+      </c>
+      <c r="D8" s="44" t="n">
+        <f aca="false">'Giả định'!$B$5</f>
+        <v>0.85</v>
+      </c>
+      <c r="E8" s="44" t="n">
+        <f aca="false">'Giả định'!$B$5</f>
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="B9" s="12" t="n">
+        <f aca="false">ROUND(B7*B8,0)</f>
+        <v>255</v>
+      </c>
+      <c r="C9" s="12" t="n">
+        <f aca="false">ROUND(C7*C8,0)</f>
+        <v>255</v>
+      </c>
+      <c r="D9" s="12" t="n">
+        <f aca="false">ROUND(D7*D8,0)</f>
+        <v>255</v>
+      </c>
+      <c r="E9" s="12" t="n">
+        <f aca="false">ROUND(E7*E8,0)</f>
+        <v>255</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="s">
+        <v>260</v>
+      </c>
+      <c r="B10" s="32" t="n">
+        <f aca="false">'Chi phí'!$E$5*'Chi phí'!$F$5+'Chi phí'!$E$6*'Chi phí'!$F$6</f>
+        <v>7000000</v>
+      </c>
+      <c r="C10" s="13" t="n">
+        <v>4200000</v>
+      </c>
+      <c r="D10" s="13" t="n">
+        <v>3300000</v>
+      </c>
+      <c r="E10" s="13" t="n">
+        <v>7000000</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="B11" s="45" t="n">
+        <f aca="false">'Giả định'!$B$19</f>
+        <v>1.4</v>
+      </c>
+      <c r="C11" s="45" t="n">
+        <f aca="false">'Giả định'!$B$19</f>
+        <v>1.4</v>
+      </c>
+      <c r="D11" s="45" t="n">
+        <f aca="false">'Giả định'!$B$19</f>
+        <v>1.4</v>
+      </c>
+      <c r="E11" s="45" t="n">
+        <f aca="false">'Giả định'!$B$19</f>
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7" t="s">
+        <v>262</v>
+      </c>
+      <c r="B12" s="32" t="n">
+        <f aca="false">'Giả định'!$B$20</f>
+        <v>500000</v>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>1450000</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>1300000</v>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>2100000</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" s="12" t="n">
+        <f aca="false">MAX('Giả định'!$B$9,ROUNDUP(B9/'Giả định'!$B$7,0)+'Giả định'!$B$8)</f>
+        <v>27</v>
+      </c>
+      <c r="C13" s="12" t="n">
+        <f aca="false">MAX('Giả định'!$B$9,ROUNDUP(C9/'Giả định'!$B$7,0)+'Giả định'!$B$8)</f>
+        <v>27</v>
+      </c>
+      <c r="D13" s="12" t="n">
+        <f aca="false">MAX('Giả định'!$B$9,ROUNDUP(D9/'Giả định'!$B$7,0)+'Giả định'!$B$8)</f>
+        <v>27</v>
+      </c>
+      <c r="E13" s="12" t="n">
+        <f aca="false">MAX('Giả định'!$B$9,ROUNDUP(E9/'Giả định'!$B$7,0)+'Giả định'!$B$8)</f>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="B16" s="12" t="n">
+        <f aca="false">(B29+B30*B13+B31*B9+'Giả định'!$B$15*(B32+B33*B13+B34*B9))*(1+'Giả định'!$B$16)</f>
+        <v>459356700</v>
+      </c>
+      <c r="C16" s="12" t="n">
+        <f aca="false">(C29+C30*C13+C31*C9+'Giả định'!$B$15*(C32+C33*C13+C34*C9))*(1+'Giả định'!$B$16)</f>
+        <v>259007100</v>
+      </c>
+      <c r="D16" s="12" t="n">
+        <f aca="false">(D29+D30*D13+D31*D9+'Giả định'!$B$15*(D32+D33*D13+D34*D9))*(1+'Giả định'!$B$16)</f>
+        <v>227733000</v>
+      </c>
+      <c r="E16" s="12" t="n">
+        <f aca="false">(E29+E30*E13+E31*E9+'Giả định'!$B$15*(E32+E33*E13+E34*E9))*(1+'Giả định'!$B$16)</f>
+        <v>356304300</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="B17" s="12" t="n">
+        <f aca="false">B9*(B12/B11+B35)+'Giả định'!$B$24</f>
+        <v>94928571.4285714</v>
+      </c>
+      <c r="C17" s="12" t="n">
+        <f aca="false">C9*(C12/C11+C35)+'Giả định'!$B$24</f>
+        <v>267964285.714286</v>
+      </c>
+      <c r="D17" s="12" t="n">
+        <f aca="false">D9*(D12/D11+D35)+'Giả định'!$B$24</f>
+        <v>240642857.142857</v>
+      </c>
+      <c r="E17" s="12" t="n">
+        <f aca="false">E9*(E12/E11+E35)+'Giả định'!$B$24</f>
+        <v>386357142.857143</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="33" t="s">
+        <v>263</v>
+      </c>
+      <c r="B18" s="28" t="n">
+        <f aca="false">B17-B16</f>
+        <v>-364428128.571429</v>
+      </c>
+      <c r="C18" s="28" t="n">
+        <f aca="false">C17-C16</f>
+        <v>8957185.71428567</v>
+      </c>
+      <c r="D18" s="28" t="n">
+        <f aca="false">D17-D16</f>
+        <v>12909857.1428571</v>
+      </c>
+      <c r="E18" s="28" t="n">
+        <f aca="false">E17-E16</f>
+        <v>30052842.8571429</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="33" t="s">
+        <v>264</v>
+      </c>
+      <c r="B19" s="46" t="str">
+        <f aca="false">IF(B18+'Giả định'!$B$29&gt;=0,"KHÔNG LỖ","LỖ "&amp;ROUND(-(B18+'Giả định'!$B$29)/1000000,0)&amp;" triệu")</f>
+        <v>LỖ 364 triệu</v>
+      </c>
+      <c r="C19" s="46" t="str">
+        <f aca="false">IF(C18+'Giả định'!$B$29&gt;=0,"KHÔNG LỖ","LỖ "&amp;ROUND(-(C18+'Giả định'!$B$29)/1000000,0)&amp;" triệu")</f>
+        <v>KHÔNG LỖ</v>
+      </c>
+      <c r="D19" s="46" t="str">
+        <f aca="false">IF(D18+'Giả định'!$B$29&gt;=0,"KHÔNG LỖ","LỖ "&amp;ROUND(-(D18+'Giả định'!$B$29)/1000000,0)&amp;" triệu")</f>
+        <v>KHÔNG LỖ</v>
+      </c>
+      <c r="E19" s="46" t="str">
+        <f aca="false">IF(E18+'Giả định'!$B$29&gt;=0,"KHÔNG LỖ","LỖ "&amp;ROUND(-(E18+'Giả định'!$B$29)/1000000,0)&amp;" triệu")</f>
+        <v>KHÔNG LỖ</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="B20" s="12" t="n">
+        <f aca="false">B12/B11+B35-((B30+'Giả định'!$B$15*B33)/'Giả định'!$B$7+B31+'Giả định'!$B$15*B34)*(1+'Giả định'!$B$16)</f>
+        <v>-581871.092436975</v>
+      </c>
+      <c r="C20" s="12" t="n">
+        <f aca="false">C12/C11+C35-((C30+'Giả định'!$B$15*C33)/'Giả định'!$B$7+C31+'Giả định'!$B$15*C34)*(1+'Giả định'!$B$16)</f>
+        <v>476640.336134454</v>
+      </c>
+      <c r="D20" s="12" t="n">
+        <f aca="false">D12/D11+D35-((D30+'Giả định'!$B$15*D33)/'Giả định'!$B$7+D31+'Giả định'!$B$15*D34)*(1+'Giả định'!$B$16)</f>
+        <v>485327.478991597</v>
+      </c>
+      <c r="E20" s="12" t="n">
+        <f aca="false">E12/E11+E35-((E30+'Giả định'!$B$15*E33)/'Giả định'!$B$7+E31+'Giả định'!$B$15*E34)*(1+'Giả định'!$B$16)</f>
+        <v>580566.050420168</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="B21" s="12" t="n">
+        <f aca="false">(B29+'Giả định'!$B$15*B32+'Giả định'!$B$8*(B30+'Giả định'!$B$15*B33))*(1+'Giả định'!$B$16)</f>
+        <v>211464000</v>
+      </c>
+      <c r="C21" s="12" t="n">
+        <f aca="false">(C29+'Giả định'!$B$15*C32+'Giả định'!$B$8*(C30+'Giả định'!$B$15*C33))*(1+'Giả định'!$B$16)</f>
+        <v>109828400</v>
+      </c>
+      <c r="D21" s="12" t="n">
+        <f aca="false">(D29+'Giả định'!$B$15*D32+'Giả định'!$B$8*(D30+'Giả định'!$B$15*D33))*(1+'Giả định'!$B$16)</f>
+        <v>108670100</v>
+      </c>
+      <c r="E21" s="12" t="n">
+        <f aca="false">(E29+'Giả định'!$B$15*E32+'Giả định'!$B$8*(E30+'Giả định'!$B$15*E33))*(1+'Giả định'!$B$16)</f>
+        <v>113432000</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="33" t="s">
+        <v>267</v>
+      </c>
+      <c r="B24" s="34" t="n">
+        <f aca="false">IF(B9=0,0,(B16-'Giả định'!$B$29-'Giả định'!$B$24-B9*B35)*B11/B9)</f>
+        <v>2500781.88235294</v>
+      </c>
+      <c r="C24" s="34" t="n">
+        <f aca="false">IF(C9=0,0,(C16-'Giả định'!$B$29-'Giả định'!$B$24-C9*C35)*C11/C9)</f>
+        <v>1400823.29411765</v>
+      </c>
+      <c r="D24" s="34" t="n">
+        <f aca="false">IF(D9=0,0,(D16-'Giả định'!$B$29-'Giả định'!$B$24-D9*D35)*D11/D9)</f>
+        <v>1229122.35294118</v>
+      </c>
+      <c r="E24" s="34" t="n">
+        <f aca="false">IF(E9=0,0,(E16-'Giả định'!$B$29-'Giả định'!$B$24-E9*E35)*E11/E9)</f>
+        <v>1935004</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="33" t="s">
+        <v>268</v>
+      </c>
+      <c r="B25" s="34" t="n">
+        <f aca="false">B10+(B18+'Giả định'!$B$29)/(B13*(1+'Giả định'!$B$15)*(1+'Giả định'!$B$16))</f>
+        <v>-3487442.18744219</v>
+      </c>
+      <c r="C25" s="34" t="n">
+        <f aca="false">C10+(C18+'Giả định'!$B$29)/(C13*(1+'Giả định'!$B$15)*(1+'Giả định'!$B$16))</f>
+        <v>4457768.15776816</v>
+      </c>
+      <c r="D25" s="34" t="n">
+        <f aca="false">D10+(D18+'Giả định'!$B$29)/(D13*(1+'Giả định'!$B$15)*(1+'Giả định'!$B$16))</f>
+        <v>3671517.37151737</v>
+      </c>
+      <c r="E25" s="34" t="n">
+        <f aca="false">E10+(E18+'Giả định'!$B$29)/(E13*(1+'Giả định'!$B$15)*(1+'Giả định'!$B$16))</f>
+        <v>7864854.89818823</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="7" t="s">
+        <v>269</v>
+      </c>
+      <c r="B26" s="12" t="str">
+        <f aca="false">IF(B20&lt;=0,"Không bao giờ",MAX(0,B21-'Giả định'!$B$24)/B20)</f>
+        <v>Không bao giờ</v>
+      </c>
+      <c r="C26" s="12" t="n">
+        <f aca="false">IF(C20&lt;=0,"Không bao giờ",MAX(0,C21-'Giả định'!$B$24)/C20)</f>
+        <v>230.421959019891</v>
+      </c>
+      <c r="D26" s="12" t="n">
+        <f aca="false">IF(D20&lt;=0,"Không bao giờ",MAX(0,D21-'Giả định'!$B$24)/D20)</f>
+        <v>223.910874005718</v>
+      </c>
+      <c r="E26" s="12" t="n">
+        <f aca="false">IF(E20&lt;=0,"Không bao giờ",MAX(0,E21-'Giả định'!$B$24)/E20)</f>
+        <v>195.381731187876</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="B28" s="6"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
+      <c r="E28" s="6"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="9" t="s">
+        <v>271</v>
+      </c>
+      <c r="B29" s="25" t="n">
+        <f aca="false">CHOOSE(B$6,'Chi phí'!$C$77,'Chi phí'!$C$78)</f>
+        <v>180500000</v>
+      </c>
+      <c r="C29" s="25" t="n">
+        <f aca="false">CHOOSE(C$6,'Chi phí'!$C$77,'Chi phí'!$C$78)</f>
+        <v>93300000</v>
+      </c>
+      <c r="D29" s="25" t="n">
+        <f aca="false">CHOOSE(D$6,'Chi phí'!$C$77,'Chi phí'!$C$78)</f>
+        <v>93300000</v>
+      </c>
+      <c r="E29" s="25" t="n">
+        <f aca="false">CHOOSE(E$6,'Chi phí'!$C$77,'Chi phí'!$C$78)</f>
+        <v>93300000</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="9" t="s">
+        <v>272</v>
+      </c>
+      <c r="B30" s="25" t="n">
+        <f aca="false">CHOOSE(B$6,'Chi phí'!$D$77,'Chi phí'!$D$78)-('Chi phí'!$J$5+'Chi phí'!$J$6)+B10</f>
+        <v>7150000</v>
+      </c>
+      <c r="C30" s="25" t="n">
+        <f aca="false">CHOOSE(C$6,'Chi phí'!$D$77,'Chi phí'!$D$78)-('Chi phí'!$J$5+'Chi phí'!$J$6)+C10</f>
+        <v>4300000</v>
+      </c>
+      <c r="D30" s="25" t="n">
+        <f aca="false">CHOOSE(D$6,'Chi phí'!$D$77,'Chi phí'!$D$78)-('Chi phí'!$J$5+'Chi phí'!$J$6)+D10</f>
+        <v>3400000</v>
+      </c>
+      <c r="E30" s="25" t="n">
+        <f aca="false">CHOOSE(E$6,'Chi phí'!$D$77,'Chi phí'!$D$78)-('Chi phí'!$J$5+'Chi phí'!$J$6)+E10</f>
+        <v>7100000</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="9" t="s">
+        <v>273</v>
+      </c>
+      <c r="B31" s="25" t="n">
+        <f aca="false">CHOOSE(B$6,'Chi phí'!$E$77,'Chi phí'!$E$78)</f>
+        <v>33400</v>
+      </c>
+      <c r="C31" s="25" t="n">
+        <f aca="false">CHOOSE(C$6,'Chi phí'!$E$77,'Chi phí'!$E$78)</f>
+        <v>20600</v>
+      </c>
+      <c r="D31" s="25" t="n">
+        <f aca="false">CHOOSE(D$6,'Chi phí'!$E$77,'Chi phí'!$E$78)</f>
+        <v>20600</v>
+      </c>
+      <c r="E31" s="25" t="n">
+        <f aca="false">CHOOSE(E$6,'Chi phí'!$E$77,'Chi phí'!$E$78)</f>
+        <v>20600</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="9" t="s">
+        <v>274</v>
+      </c>
+      <c r="B32" s="25" t="n">
+        <f aca="false">CHOOSE(B$6,'Chi phí'!$F$77,'Chi phí'!$F$78)</f>
+        <v>20000000</v>
+      </c>
+      <c r="C32" s="25" t="n">
+        <f aca="false">CHOOSE(C$6,'Chi phí'!$F$77,'Chi phí'!$F$78)</f>
+        <v>9000000</v>
+      </c>
+      <c r="D32" s="25" t="n">
+        <f aca="false">CHOOSE(D$6,'Chi phí'!$F$77,'Chi phí'!$F$78)</f>
+        <v>9000000</v>
+      </c>
+      <c r="E32" s="25" t="n">
+        <f aca="false">CHOOSE(E$6,'Chi phí'!$F$77,'Chi phí'!$F$78)</f>
+        <v>9000000</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="9" t="s">
+        <v>275</v>
+      </c>
+      <c r="B33" s="25" t="n">
+        <f aca="false">CHOOSE(B$6,'Chi phí'!$G$77,'Chi phí'!$G$78)-('Chi phí'!$J$5*'Chi phí'!$G$5+'Chi phí'!$J$6*'Chi phí'!$G$6)+B10</f>
+        <v>7000000</v>
+      </c>
+      <c r="C33" s="25" t="n">
+        <f aca="false">CHOOSE(C$6,'Chi phí'!$G$77,'Chi phí'!$G$78)-('Chi phí'!$J$5*'Chi phí'!$G$5+'Chi phí'!$J$6*'Chi phí'!$G$6)+C10</f>
+        <v>4200000</v>
+      </c>
+      <c r="D33" s="25" t="n">
+        <f aca="false">CHOOSE(D$6,'Chi phí'!$G$77,'Chi phí'!$G$78)-('Chi phí'!$J$5*'Chi phí'!$G$5+'Chi phí'!$J$6*'Chi phí'!$G$6)+D10</f>
+        <v>3300000</v>
+      </c>
+      <c r="E33" s="25" t="n">
+        <f aca="false">CHOOSE(E$6,'Chi phí'!$G$77,'Chi phí'!$G$78)-('Chi phí'!$J$5*'Chi phí'!$G$5+'Chi phí'!$J$6*'Chi phí'!$G$6)+E10</f>
+        <v>7000000</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="9" t="s">
+        <v>276</v>
+      </c>
+      <c r="B34" s="25" t="n">
+        <f aca="false">CHOOSE(B$6,'Chi phí'!$H$77,'Chi phí'!$H$78)</f>
+        <v>0</v>
+      </c>
+      <c r="C34" s="25" t="n">
+        <f aca="false">CHOOSE(C$6,'Chi phí'!$H$77,'Chi phí'!$H$78)</f>
+        <v>0</v>
+      </c>
+      <c r="D34" s="25" t="n">
+        <f aca="false">CHOOSE(D$6,'Chi phí'!$H$77,'Chi phí'!$H$78)</f>
+        <v>0</v>
+      </c>
+      <c r="E34" s="25" t="n">
+        <f aca="false">CHOOSE(E$6,'Chi phí'!$H$77,'Chi phí'!$H$78)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="9" t="s">
+        <v>277</v>
+      </c>
+      <c r="B35" s="25" t="n">
+        <f aca="false">(B9*0+(1-B8)/B8*'Giả định'!$B$21*'Giả định'!$B$22/B11)</f>
+        <v>15126.0504201681</v>
+      </c>
+      <c r="C35" s="25" t="n">
+        <f aca="false">(C9*0+(1-C8)/C8*'Giả định'!$B$21*'Giả định'!$B$22/C11)</f>
+        <v>15126.0504201681</v>
+      </c>
+      <c r="D35" s="25" t="n">
+        <f aca="false">(D9*0+(1-D8)/D8*'Giả định'!$B$21*'Giả định'!$B$22/D11)</f>
+        <v>15126.0504201681</v>
+      </c>
+      <c r="E35" s="25" t="n">
+        <f aca="false">(E9*0+(1-E8)/E8*'Giả định'!$B$21*'Giả định'!$B$22/E11)</f>
+        <v>15126.0504201681</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="9" t="s">
+        <v>278</v>
+      </c>
+      <c r="B37" s="9" t="str">
+        <f aca="false">IF(ABS(B16-'Hòa vốn'!B8)&lt;1,"OK","LỆCH")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="41" t="s">
+        <v>279</v>
+      </c>
+      <c r="B38" s="41"/>
+      <c r="C38" s="41"/>
+      <c r="D38" s="41"/>
+      <c r="E38" s="41"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A38:E38"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B19:E19">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+      <formula>"KHÔNG LỖ"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B18:E18">
+    <cfRule type="cellIs" priority="3" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B6:E6" type="list">
+      <formula1>"1,2"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:K1005"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -6994,47 +8166,47 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>238</v>
+        <v>280</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>239</v>
+        <v>281</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>240</v>
+        <v>282</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>241</v>
+        <v>283</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>242</v>
+        <v>284</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>243</v>
+        <v>285</v>
       </c>
       <c r="G4" s="18" t="s">
-        <v>244</v>
+        <v>286</v>
       </c>
       <c r="H4" s="18" t="s">
-        <v>245</v>
+        <v>287</v>
       </c>
       <c r="I4" s="18" t="s">
-        <v>246</v>
+        <v>288</v>
       </c>
       <c r="J4" s="18" t="s">
-        <v>247</v>
+        <v>289</v>
       </c>
       <c r="K4" s="18" t="s">
-        <v>248</v>
+        <v>290</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>